<commit_message>
docs: update changelog with Tebex coupons, search bars, and security audit
</commit_message>
<xml_diff>
--- a/docs/session-changelog.xlsx
+++ b/docs/session-changelog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Clients\Priyam\FiveCrux\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7089D241-3098-4D5A-9A0F-8DE9C62406DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC28C77E-5298-49B6-8930-371C3EEC671B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{E9E1534B-C991-495F-AE32-06FC689859A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E9E1534B-C991-495F-AE32-06FC689859A5}"/>
   </bookViews>
   <sheets>
     <sheet name="Fixes &amp; Changes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="135">
   <si>
     <t>FiveCrux  -  Website Fixes &amp; Changes</t>
   </si>
@@ -390,7 +390,46 @@
     <t>Generated the missing migration for local testing. Confirmed (read-only) production already has the column, so no prod action is needed.</t>
   </si>
   <si>
-    <t>44 items  -  12 Features  -  21 Bug Fixes  -  11 Improvements</t>
+    <t>Coupons/Creator Codes management lived on FiveCrux's own database, disconnected from the real Tebex checkout.</t>
+  </si>
+  <si>
+    <t>Switched coupon validation to check directly against Tebex; removed the now-redundant local coupon/creator-code management from the profile (kept in code, just disabled, in case it's needed again).</t>
+  </si>
+  <si>
+    <t>Ad Slots</t>
+  </si>
+  <si>
+    <t>The 'Create New Ad' and file-upload forms still used an old grey theme that didn't match the rest of the site.</t>
+  </si>
+  <si>
+    <t>Rethemed both forms (and the Props tab cards) to the site's black/orange look.</t>
+  </si>
+  <si>
+    <t>Admin Dashboard</t>
+  </si>
+  <si>
+    <t>Admins had no way to search or filter the Assets/Props/Giveaways/Ads lists in the admin dashboard - had to scroll through everything.</t>
+  </si>
+  <si>
+    <t>Added a search box plus category/status filters to all four admin dashboard tabs, and to the profile's Props tab.</t>
+  </si>
+  <si>
+    <t>The 'Buy Slot' cards under My Ad Slots &gt; Featured Scripts used a mismatched purple/pink color scheme, unlike every other tab.</t>
+  </si>
+  <si>
+    <t>Rethemed to the site's orange, matching Ads/Props/Assets.</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>A full security audit found several ways a logged-in account could act outside its own listings: edit or delete another seller's script/giveaway, mark a giveaway as 'Featured' for free, create an ad slot without actually buying one, or inflate giveaway-entry points by faking a Discord-join.</t>
+  </si>
+  <si>
+    <t>Closed all of the above: ownership checks added everywhere they were missing, 'Featured' is now admin-only, ad/slot purchases are verified server-side, and Discord-join claims are re-checked before awarding points.</t>
+  </si>
+  <si>
+    <t>49 items  -  13 Features  -  24 Bug Fixes  -  12 Improvements</t>
   </si>
 </sst>
 </file>
@@ -645,18 +684,6 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -689,6 +716,18 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2259,7 +2298,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F609A6-E1DC-48C7-B847-60D5C7C74FFA}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" customWidth="1"/>
@@ -2271,40 +2310,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
+      <c r="A3" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -3213,22 +3252,22 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="24">
+      <c r="A40" s="20">
         <v>36</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D40" s="26" t="s">
+      <c r="D40" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="F40" s="27" t="s">
+      <c r="F40" s="23" t="s">
         <v>14</v>
       </c>
       <c r="G40" s="13" t="s">
@@ -3239,110 +3278,110 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="29">
+      <c r="A41" s="25">
         <v>37</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="30" t="s">
+      <c r="C41" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="31" t="s">
+      <c r="D41" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="31" t="s">
+      <c r="E41" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="F41" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
+      <c r="F41" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" s="24"/>
+      <c r="H41" s="24"/>
     </row>
     <row r="42" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="24">
+      <c r="A42" s="20">
         <v>38</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="30" t="s">
+      <c r="C42" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D42" s="26" t="s">
+      <c r="D42" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="E42" s="26" t="s">
+      <c r="E42" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="F42" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
+      <c r="F42" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" s="19"/>
+      <c r="H42" s="19"/>
     </row>
     <row r="43" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="29">
+      <c r="A43" s="25">
         <v>39</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="30" t="s">
+      <c r="C43" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D43" s="32" t="s">
+      <c r="D43" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="31" t="s">
+      <c r="E43" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="F43" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
+      <c r="F43" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="24">
+      <c r="A44" s="20">
         <v>40</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C44" s="33" t="s">
+      <c r="C44" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="F44" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
+      <c r="F44" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" s="19"/>
+      <c r="H44" s="19"/>
     </row>
     <row r="45" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="29">
+      <c r="A45" s="25">
         <v>41</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C45" s="25" t="s">
+      <c r="C45" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D45" s="31" t="s">
+      <c r="D45" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="E45" s="31" t="s">
+      <c r="E45" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="F45" s="27" t="s">
+      <c r="F45" s="23" t="s">
         <v>14</v>
       </c>
       <c r="G45" s="8" t="s">
@@ -3353,22 +3392,22 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="24">
+      <c r="A46" s="20">
         <v>42</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="C46" s="33" t="s">
+      <c r="C46" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="D46" s="26" t="s">
+      <c r="D46" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="E46" s="26" t="s">
+      <c r="E46" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="F46" s="27" t="s">
+      <c r="F46" s="23" t="s">
         <v>14</v>
       </c>
       <c r="G46" s="13" t="s">
@@ -3379,50 +3418,180 @@
       </c>
     </row>
     <row r="47" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="29">
+      <c r="A47" s="25">
         <v>43</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C47" s="25" t="s">
+      <c r="C47" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D47" s="32" t="s">
+      <c r="D47" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="E47" s="31" t="s">
+      <c r="E47" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="F47" s="30" t="s">
+      <c r="F47" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="G47" s="28"/>
-      <c r="H47" s="28"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="24"/>
     </row>
     <row r="48" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="24">
+      <c r="A48" s="20">
         <v>44</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C48" s="25" t="s">
+      <c r="C48" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D48" s="26" t="s">
+      <c r="D48" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="F48" s="27" t="s">
+      <c r="F48" s="23" t="s">
         <v>14</v>
       </c>
       <c r="G48" s="13" t="s">
         <v>15</v>
       </c>
       <c r="H48" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A49" s="25">
+        <v>45</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D49" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="E49" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="F49" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G49" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A50" s="20">
+        <v>46</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="E50" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F50" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A51" s="25">
+        <v>47</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C51" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="E51" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F51" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A52" s="20">
+        <v>48</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="E52" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="F52" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="25">
+        <v>49</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C53" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="E53" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="F53" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H53" s="24" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>